<commit_message>
Ejemplos realistas del manifiesto, PCE realista y PDF de servidor con Docker
- ejemplos_manifiesto: el ejercicio modelo y los papeles de muestra se arman con
  los MISMOS archivos que el cliente descarga con «↓ Ejemplo» (lector del ciclo +
  mapeo automático), no con los escenarios mínimos de prueba.
- PCE: ejemplo realista desde la misma cartera ficticia de pérdidas incurridas
  (6 clientes, 2024 y 2025, castigos coherentes, provisión registrada = la de PI).
- papeles_muestra.py: las 20 herramientas (incluye PI y PCE) con INDICE.html.
- PDF de servidor: render.yaml pasa el servicio a runtime Docker
  (Dockerfile.render: python:3.12-slim + requirements-prod + WeasyPrint y sus
  librerías nativas); .dockerignore conserva ejemplos y manifiesto.
- graficos_svg: barras 3D, barras + línea, líneas, área, puntos y dona (WIP).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KenmW9mmzjSrfJfKBkhhtH
</commit_message>
<xml_diff>
--- a/frontend/public/ejemplos/pce_simplificada_niif9/RQ-001_actual.xlsx
+++ b/frontend/public/ejemplos/pce_simplificada_niif9/RQ-001_actual.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,52 +457,542 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>F-10</t>
+          <t>001-001-000001009</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Vialidad Norte S.A.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>15/11/2024</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+          <t>04/10/2023</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2266.21</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1090044556001</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>F-20</t>
+          <t>001-001-000001011</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Obras Civiles Pacífico S.A.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>15/11/2025</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
+          <t>05/05/2023</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4342.93</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1390066778001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>001-001-000001021</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Minera Austral S.A.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>05/04/2024</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1375.09</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1790033445001</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>001-001-000001022</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Vialidad Norte S.A.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>12/04/2024</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>7172.35</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1090044556001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>001-001-000001023</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Hidrosur Cía. Ltda.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>06/10/2024</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1787.01</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0190055667001</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>001-001-000001024</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Obras Civiles Pacífico S.A.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>25/11/2024</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5514.61</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1390066778001</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>001-001-000001027</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Minera Austral S.A.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>15/11/2024</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>442.06</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1790033445001</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>001-001-000001028</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Vialidad Norte S.A.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>23/05/2024</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8659.559999999999</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1090044556001</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>001-001-000001029</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Vialidad Norte S.A.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>01/01/2026</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>7754.65</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1090044556001</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>001-001-000001030</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Hidrosur Cía. Ltda.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>29394.77</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0190055667001</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>001-001-000001031</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Obras Civiles Pacífico S.A.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>7119.93</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1390066778001</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>001-001-000001032</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Constructora Andina S.A.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>27/01/2026</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>28854.13</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1790011223001</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>001-001-000001033</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Agroexport del Litoral Cía. Ltda.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>07/12/2025</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>27938.78</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0990022334001</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>001-001-000001034</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Minera Austral S.A.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>03/02/2026</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>17253.71</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1790033445001</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>001-001-000001035</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vialidad Norte S.A.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>05/10/2025</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2101.88</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1090044556001</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>001-001-000001036</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Hidrosur Cía. Ltda.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>11/10/2025</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5870.86</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0190055667001</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>001-001-000001037</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Obras Civiles Pacífico S.A.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>16/10/2025</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1277.27</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1390066778001</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>001-001-000001040</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Minera Austral S.A.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>22/10/2025</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>4403.3</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1790033445001</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>001-001-000001041</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Vialidad Norte S.A.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>04/05/2025</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2839.34</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>1090044556001</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>001-001-000001042</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hidrosur Cía. Ltda.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>691.42</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0190055667001</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>